<commit_message>
implementacion algoritmo genetico en geomip
</commit_message>
<xml_diff>
--- a/GeoMIP/results/resultados_N3A.xlsx
+++ b/GeoMIP/results/resultados_N3A.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,40 +429,45 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Estado Inicial</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Alcance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Mecanismo</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Pérdida</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tiempo (s)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Tiempo Real (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Partición</t>
         </is>
@@ -477,39 +482,42 @@
       <c r="B2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.25</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.002805948257446289</v>
-      </c>
       <c r="I2" t="n">
-        <v>0.01222658157348633</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>|  A,C  || B |
-| a,b,c || ∅ |</t>
+        <v>0.002105236053466797</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.006489753723144531</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>|   ∅   || A,C |
+| a,b,c ||  ∅  |</t>
         </is>
       </c>
     </row>
@@ -522,39 +530,42 @@
       <c r="B3" t="n">
         <v>3</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>0.25</v>
-      </c>
       <c r="H3" t="n">
-        <v>0.002483129501342773</v>
+        <v>0.75</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01089382171630859</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>|  A,C  || B |
-| a,b,c || ∅ |</t>
+        <v>0.00249028205871582</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.006489753723144531</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>|   ∅   || A,B,C || ∅ |
+| a,b,c ||   ∅   || ∅ |</t>
         </is>
       </c>
     </row>

</xml_diff>